<commit_message>
[add] added bkr summary in mode share
</commit_message>
<xml_diff>
--- a/inputs/model/CatVarDict_2023.xlsx
+++ b/inputs/model/CatVarDict_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\BKR3-24-v1\inputs\model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\BKRCast\BKR3-24-v1\inputs\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B0494D-39E7-4840-A0F6-9AD3CD6D7CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5E10F3-7E2B-43CA-98D9-99C4D6F9F9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Household" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
[update] added district flow summary. #166. #173. Resolved #173.
</commit_message>
<xml_diff>
--- a/inputs/model/CatVarDict_2023.xlsx
+++ b/inputs/model/CatVarDict_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\BKRCast\BKR3-24-v1\inputs\model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\BKRCast\BKRCast\inputs\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5E10F3-7E2B-43CA-98D9-99C4D6F9F9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DC6F65-958E-409A-9174-8A9F196F28BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11370" yWindow="1470" windowWidth="15600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Household" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,25 @@
     <sheet name="Tour" sheetId="5" r:id="rId4"/>
     <sheet name="Trip" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="123">
   <si>
     <t>hownrent</t>
   </si>
@@ -387,6 +400,12 @@
   </si>
   <si>
     <t>TNC</t>
+  </si>
+  <si>
+    <t>Transit Walk Access</t>
+  </si>
+  <si>
+    <t>Transit Auto Access</t>
   </si>
 </sst>
 </file>
@@ -1523,7 +1542,7 @@
         <v>6</v>
       </c>
       <c r="H7" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -1543,7 +1562,7 @@
         <v>7</v>
       </c>
       <c r="H8" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="I8">
         <v>6</v>

</xml_diff>